<commit_message>
Drop leading 0 from day/month & fix basisOfRecord
</commit_message>
<xml_diff>
--- a/config/col-map.xlsx
+++ b/config/col-map.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gunet-my.sharepoint.com/personal/maria_prager_bioenv_gu_se/Documents/Herbarium-GB/HBGB-data/HerbariumGB-to-GBIF/v-1-11/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xpragm/code/github/herbarium-data/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="281" documentId="8_{403486E7-91D4-EC44-9677-B904FC45F416}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D613AFF-D6E6-D14B-BF54-26115972D88F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD7A3AB-9847-9242-9535-D9A5EB8F6675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8580" yWindow="8400" windowWidth="32680" windowHeight="21180" xr2:uid="{D7E58C6B-DDB6-5645-A07F-3DEAF917B064}"/>
+    <workbookView xWindow="8580" yWindow="7620" windowWidth="32680" windowHeight="21180" xr2:uid="{D7E58C6B-DDB6-5645-A07F-3DEAF917B064}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -339,9 +339,6 @@
     <t>ScientificName</t>
   </si>
   <si>
-    <t>Preserved specimen</t>
-  </si>
-  <si>
     <t>Institutioncode</t>
   </si>
   <si>
@@ -370,6 +367,9 @@
   </si>
   <si>
     <t>Uses RUBIN</t>
+  </si>
+  <si>
+    <t>PreservedSpecimen</t>
   </si>
 </sst>
 </file>
@@ -780,7 +780,7 @@
         <v>63</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -796,7 +796,7 @@
         <v>65</v>
       </c>
       <c r="C4" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -809,10 +809,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" t="s">
         <v>103</v>
-      </c>
-      <c r="C6" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -934,7 +934,7 @@
         <v>98</v>
       </c>
       <c r="D22" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -942,15 +942,15 @@
         <v>97</v>
       </c>
       <c r="D23" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D24" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
@@ -958,7 +958,7 @@
         <v>81</v>
       </c>
       <c r="D25" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
@@ -966,7 +966,7 @@
         <v>79</v>
       </c>
       <c r="D26" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -974,31 +974,31 @@
         <v>80</v>
       </c>
       <c r="D27" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D28" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D29" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>108</v>
+      </c>
+      <c r="D30" t="s">
         <v>109</v>
-      </c>
-      <c r="D30" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
@@ -1234,7 +1234,7 @@
         <v>66</v>
       </c>
       <c r="F5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G5" t="s">
         <v>67</v>
@@ -1333,19 +1333,19 @@
         <v>92</v>
       </c>
       <c r="AM5" t="s">
+        <v>104</v>
+      </c>
+      <c r="AN5" t="s">
         <v>105</v>
       </c>
-      <c r="AN5" t="s">
+      <c r="AO5" t="s">
         <v>106</v>
       </c>
-      <c r="AO5" t="s">
+      <c r="AP5" t="s">
         <v>107</v>
       </c>
-      <c r="AP5" t="s">
+      <c r="AQ5" t="s">
         <v>108</v>
-      </c>
-      <c r="AQ5" t="s">
-        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>